<commit_message>
fix(academia): carrossel de fotos NAO vira shop -> Slideshow em VIDEO + regra da sacolinha
- Photo mode/carrossel removido (nao leva sacolinha = nao vira shop)
- vira 'Slideshow em video' (fotos editadas como VIDEO no CapCut)
- aviso: so VIDEO tem sacolinha; template xlsx + plano atualizados

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rhode-vercel/public/downloads/rhode-calendario-editorial.xlsx
+++ b/rhode-vercel/public/downloads/rhode-calendario-editorial.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,11 @@
     <font>
       <b val="1"/>
       <color rgb="0017151B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FE2C55"/>
       <sz val="11"/>
     </font>
     <font>
@@ -95,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -109,13 +114,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -484,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -508,57 +516,64 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Pra bater 5 sem queimar: 3 formatos ⚡ RÁPIDOS + 2 de 🎬 PRODUÇÃO por semana.</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ SÓ VÍDEO VIRA SHOP (tem sacolinha). Carrossel de fotos NÃO leva sacolinha — se usar fotos, monta como VÍDEO (slideshow no CapCut).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Os rápidos (POV texto na tela, Photo mode) você grava vários numa tarde só.</t>
+          <t>Pra bater 5 sem queimar: 3 formatos ⚡ RÁPIDOS + 2 de 🎬 PRODUÇÃO por semana.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Os rápidos (POV texto na tela, Slideshow em vídeo, Contraste) você grava vários numa tarde.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Como usar:</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>1) Aba 'Calendário editorial' — já vem com 3 semanas x 5 vídeos preenchidas. Edita o formato, o SKU e o gancho de cada dia. Marca o status conforme grava e publica.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2) Aba 'Plano de teste' — pega 1 vídeo campeão e multiplica: mantém a estrutura, troca só o hook, e vê qual variação repete o resultado. Dobra na vencedora.</t>
+          <t>1) Aba 'Calendário editorial' — 3 semanas x 5 vídeos preenchidas. Edita formato, SKU e gancho. Marca o status conforme grava/publica.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>3) Regra de ouro do hook: o ÂNGULO é compartilhado, a FRASE é sua. Nunca copia igual — remodela na sua voz.</t>
+          <t>2) Aba 'Plano de teste' — pega 1 vídeo campeão e multiplica: mantém a estrutura, troca só o hook, dobra na variação que repetir o resultado.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>3) Regra do hook: o ÂNGULO é compartilhado, a FRASE é sua. Nunca copia igual — remodela na sua voz.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Os 12 formatos (⚡ = rápido/volume): POV texto ⚡ · Photo mode ⚡ · Contraste ⚡ · 3 looks ⚡ · Transição no beat ⚡ · GRWM · Try-on · Unboxing · Antes/depois · Conforto · Review · Restock.</t>
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Os 12 formatos (⚡=rápido/volume): POV texto ⚡ · Slideshow em vídeo ⚡ · Contraste ⚡ · 3 looks ⚡ · Transição no beat ⚡ · GRWM · Try-on · Unboxing · Antes/depois · Conforto · Review · Restock.</t>
         </is>
       </c>
     </row>
@@ -586,493 +601,493 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Semana</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Dia</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Formato</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Produto (SKU)</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Gancho (0-3s, sua voz)</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Publicado?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Semana 1 · aquecer</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Seg</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>POV texto ⚡</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>POV: a calça mais viralizada do TikTok</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr"/>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr"/>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr"/>
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Ter</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Photo mode ⚡</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Slideshow vídeo ⚡</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>3 looks que eu faria com essa calça</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr"/>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Qua</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Contraste ⚡</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>de básica a arrumada num corte</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr"/>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Qui</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Unboxing</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>chegou a calça que tá bombando</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr"/>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Sex</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Try-on</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>1,60m, veste 38 — olha o caimento</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Semana 2 · converter</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Seg</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>3 looks ⚡</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>REF525</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>1 calça, 3 looks</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr"/>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Ter</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>POV texto ⚡</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>REF525</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>POV: achei o jeans que fecha no quadril</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Qua</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Try-on/tamanho</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>REF525</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>descobre seu número em 10s</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr"/>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Qui</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Antes/depois</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>REF588</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>troquei minha calça velha por essa</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr"/>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Sex</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Conforto</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>REF588</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>senta, levanta, agacha — não marca</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Semana 3 · escalar</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Seg</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Transição ⚡</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>REF562</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>espera o look final</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr"/>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Ter</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Photo mode ⚡</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Slideshow vídeo ⚡</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>a calça que eu vivo dentro</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr"/>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Qua</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Contraste ⚡</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>REF525</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>de básica a estilosa num corte</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr"/>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr"/>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Qui</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>REF588</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>a real depois de 1 semana</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Sex</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Restock</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>voltou o estoque, corre</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>A gravar</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>A gravar</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"POV texto ⚡,Photo mode ⚡,Contraste ⚡,3 looks ⚡,Transição ⚡,GRWM,Try-on,Unboxing,Antes/depois,Conforto,Review,Restock"</formula1>
+      <formula1>"POV texto ⚡,Slideshow vídeo ⚡,Contraste ⚡,3 looks ⚡,Transição ⚡,GRWM,Try-on,Unboxing,Antes/depois,Conforto,Review,Restock"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A gravar,Gravado,Publicado"</formula1>
@@ -1105,166 +1120,166 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Campeão base (link/nome)</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>O que MANTENHO</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Variável que TROCO</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Hipótese</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Views</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Vendas</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Repetiu? (dobrar/descartar)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>(cole o link do seu campeão)</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>estrutura + ângulo + som</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>só a frase de abertura</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>novo hook segura mais nos 2s?</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr"/>
+      <c r="F2" s="8" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr"/>
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>(dobra se repetir o resultado)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
+      <c r="A3" s="9" t="n"/>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n"/>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
+      <c r="A4" s="9" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="9" t="n"/>
+      <c r="E4" s="9" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
+      <c r="A5" s="9" t="n"/>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
+      <c r="A6" s="9" t="n"/>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n"/>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="9" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>